<commit_message>
Terminado nuevo formato de pagaré
</commit_message>
<xml_diff>
--- a/public/report_templates/creditos/reportes/rptFichaCredito.xlsx
+++ b/public/report_templates/creditos/reportes/rptFichaCredito.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CredipymeApp\public\report_templates\creditos\reportes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CredypymeApp\public\report_templates\creditos\reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9551B9A2-1E48-476B-A4FA-EB372E28BEFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5FA61F-9865-41DD-966F-54F6F265D45A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2865" yWindow="1875" windowWidth="21600" windowHeight="11295" xr2:uid="{D483FF64-B468-47D6-B072-AAF7CB972AD6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D483FF64-B468-47D6-B072-AAF7CB972AD6}"/>
   </bookViews>
   <sheets>
     <sheet name="rptFichaCredito" sheetId="1" r:id="rId1"/>
@@ -154,18 +154,6 @@
     <t>Considerado 1</t>
   </si>
   <si>
-    <t>Firma FIADOR</t>
-  </si>
-  <si>
-    <t>Firma PARIENTE de FIADOR</t>
-  </si>
-  <si>
-    <t>DATOS - FIADOR</t>
-  </si>
-  <si>
-    <t>DATOS - PARIENTE DE FIADOR</t>
-  </si>
-  <si>
     <t>DATOS - TITULAR</t>
   </si>
   <si>
@@ -176,6 +164,18 @@
   </si>
   <si>
     <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>DATOS - AVAL</t>
+  </si>
+  <si>
+    <t>DATOS - PARIENTE DE AVAL</t>
+  </si>
+  <si>
+    <t>Firma AVAL</t>
+  </si>
+  <si>
+    <t>Firma PARIENTE de AVAL</t>
   </si>
 </sst>
 </file>
@@ -480,44 +480,44 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -873,12 +873,12 @@
     </row>
     <row r="2" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="11"/>
       <c r="G2" s="12" t="s">
         <v>2</v>
@@ -905,19 +905,19 @@
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
+      <c r="G4" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -934,11 +934,11 @@
       <c r="G5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="H5" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="32"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1099,36 +1099,36 @@
     </row>
     <row r="14" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="6"/>
-      <c r="G14" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
+      <c r="G14" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
+      <c r="B15" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
       <c r="F15" s="6"/>
-      <c r="G15" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="H15" s="32"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="32"/>
+      <c r="G15" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1306,34 +1306,34 @@
     </row>
     <row r="25" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
+      <c r="B25" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="6"/>
-      <c r="G25" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="37"/>
+      <c r="G25" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34"/>
       <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="30"/>
       <c r="K26" s="2"/>
     </row>
     <row r="27" spans="1:11" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1426,29 +1426,29 @@
       <c r="B32" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="33" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="34"/>
+      <c r="C32" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="38"/>
       <c r="K32" s="2"/>
     </row>
     <row r="33" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
+      <c r="C33" s="30"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
       <c r="I33" s="8" t="s">
         <v>17</v>
       </c>
@@ -1462,16 +1462,16 @@
       <c r="B34" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="31"/>
+      <c r="C34" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:11" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1496,7 +1496,7 @@
         <v>38</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="J35" s="26"/>
       <c r="K35" s="2"/>
@@ -1574,15 +1574,15 @@
     </row>
     <row r="39" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
-      <c r="B39" s="32" t="s">
+      <c r="B39" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
       <c r="I39" s="8" t="s">
         <v>17</v>
       </c>
@@ -1710,30 +1710,30 @@
     </row>
     <row r="45" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="32"/>
-      <c r="J45" s="32"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
+      <c r="E45" s="30"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
+      <c r="J45" s="30"/>
       <c r="K45" s="2"/>
     </row>
     <row r="46" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
-      <c r="B46" s="39"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39"/>
-      <c r="J46" s="39"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="31"/>
+      <c r="F46" s="31"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="31"/>
+      <c r="J46" s="31"/>
       <c r="K46" s="2"/>
     </row>
     <row r="47" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1798,17 +1798,17 @@
     </row>
     <row r="51" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
-      <c r="B51" s="38" t="s">
+      <c r="B51" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C51" s="38"/>
-      <c r="D51" s="38"/>
-      <c r="E51" s="38"/>
-      <c r="F51" s="38"/>
-      <c r="G51" s="38"/>
-      <c r="H51" s="38"/>
-      <c r="I51" s="38"/>
-      <c r="J51" s="38"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="27"/>
+      <c r="I51" s="27"/>
+      <c r="J51" s="27"/>
       <c r="K51" s="2"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
@@ -1826,6 +1826,45 @@
     </row>
   </sheetData>
   <mergeCells count="55">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="C12:J12"/>
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="C11:J11"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="C31:J31"/>
+    <mergeCell ref="C32:J32"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C24:J24"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="C28:J28"/>
+    <mergeCell ref="C29:J29"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="B49:H50"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="C16:E16"/>
     <mergeCell ref="B51:J51"/>
     <mergeCell ref="H16:J16"/>
     <mergeCell ref="H17:J17"/>
@@ -1842,45 +1881,6 @@
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="G25:J25"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="B49:H50"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="C30:J30"/>
-    <mergeCell ref="C31:J31"/>
-    <mergeCell ref="C32:J32"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C24:J24"/>
-    <mergeCell ref="B26:J26"/>
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="C28:J28"/>
-    <mergeCell ref="C29:J29"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="C11:J11"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="H9:J9"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.23622047244094491" top="0.23622047244094491" bottom="0.11811023622047245" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="32" orientation="portrait" r:id="rId1"/>

</xml_diff>